<commit_message>
chore: update multiple project files
</commit_message>
<xml_diff>
--- a/data/input/common/medidoralimentador/medidoralimentador.xlsx
+++ b/data/input/common/medidoralimentador/medidoralimentador.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\ELDICA\RECYM\data\input\common\medidoralimentador\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2A395D4-5DC7-4FFF-A3FB-0D02BF94B56A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB03DE83-0666-43EF-8FDD-5B65D28DE93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0537D3D3-A7EC-4918-978F-ABDC6DEFE1BE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="176">
   <si>
     <t>Medidor</t>
   </si>
@@ -291,12 +291,288 @@
   </si>
   <si>
     <t>siglas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-6603   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-6604   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-PNB6T2 </t>
+  </si>
+  <si>
+    <t>PN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-PN1T2  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-PN2T2  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-PN6T1  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-PN1T1  </t>
+  </si>
+  <si>
+    <t>PN101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PN111  </t>
+  </si>
+  <si>
+    <t>PN102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PN112  </t>
+  </si>
+  <si>
+    <t>PN103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PN113  </t>
+  </si>
+  <si>
+    <t>PN104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PN114  </t>
+  </si>
+  <si>
+    <t>PN105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PN115  </t>
+  </si>
+  <si>
+    <t>PN106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PN116  </t>
+  </si>
+  <si>
+    <t>PN107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PN117  </t>
+  </si>
+  <si>
+    <t>PN209</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PN209  </t>
+  </si>
+  <si>
+    <t>L-6117_PE</t>
+  </si>
+  <si>
+    <t>L-6613_PE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-PE6T1  </t>
+  </si>
+  <si>
+    <t>PE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barra CT </t>
+  </si>
+  <si>
+    <t>CT_PEDREG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-PE1T1  </t>
+  </si>
+  <si>
+    <t>PE101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PE121  </t>
+  </si>
+  <si>
+    <t>PE102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PE122  </t>
+  </si>
+  <si>
+    <t>PE103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PE123  </t>
+  </si>
+  <si>
+    <t>PE105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PE125  </t>
+  </si>
+  <si>
+    <t>PE104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-PE104  </t>
+  </si>
+  <si>
+    <t>PE106</t>
+  </si>
+  <si>
+    <t>PE107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-TM6T1  </t>
+  </si>
+  <si>
+    <t>TM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-TM1T1  </t>
+  </si>
+  <si>
+    <t>TM101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-TM141  </t>
+  </si>
+  <si>
+    <t>TM102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-TM142  </t>
+  </si>
+  <si>
+    <t>TM103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-TM143  </t>
+  </si>
+  <si>
+    <t>TM104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-TM144  </t>
+  </si>
+  <si>
+    <t>TM105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-TM145  </t>
+  </si>
+  <si>
+    <t>TM106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-TM146  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAB6T2   </t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAB1T2   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAB2T2   </t>
+  </si>
+  <si>
+    <t>CA206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-CA6T1  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-CA1T1  </t>
+  </si>
+  <si>
+    <t>CA101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CA131  </t>
+  </si>
+  <si>
+    <t>CA103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CA133  </t>
+  </si>
+  <si>
+    <t>CA104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CA134  </t>
+  </si>
+  <si>
+    <t>CA105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-CA135  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMB6T2   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMB1T2   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">L6603-02 </t>
+  </si>
+  <si>
+    <t>L6619</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-6618   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">L6619 </t>
+  </si>
+  <si>
+    <t>L-6613</t>
+  </si>
+  <si>
+    <t>L-6116</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHNB1T1  </t>
+  </si>
+  <si>
+    <t>CHN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHNB2T1  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHNB6T1  </t>
+  </si>
+  <si>
+    <t>CHN101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHN101   </t>
+  </si>
+  <si>
+    <t>CHN102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHN102   </t>
+  </si>
+  <si>
+    <t>CHN201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHN201   </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -372,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -402,6 +678,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -736,10 +1021,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{316871D9-CF50-4EFA-B4A9-0D945CB9EBBB}">
-  <dimension ref="A2:D52"/>
+  <dimension ref="A2:D112"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
@@ -1392,6 +1678,824 @@
       <c r="C52" s="9"/>
       <c r="D52" s="9"/>
     </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B53" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="C53" s="12">
+        <v>60</v>
+      </c>
+      <c r="D53" s="11"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B54" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C54" s="12">
+        <v>60</v>
+      </c>
+      <c r="D54" s="11"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="C55" s="12">
+        <v>60</v>
+      </c>
+      <c r="D55" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="C56" s="12">
+        <v>10</v>
+      </c>
+      <c r="D56" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="C57" s="13">
+        <v>22.9</v>
+      </c>
+      <c r="D57" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B58" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C58" s="12">
+        <v>60</v>
+      </c>
+      <c r="D58" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B59" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C59" s="12">
+        <v>10</v>
+      </c>
+      <c r="D59" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="C60" s="12">
+        <v>10</v>
+      </c>
+      <c r="D60" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B61" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C61" s="12">
+        <v>10</v>
+      </c>
+      <c r="D61" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B62" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="C62" s="12">
+        <v>10</v>
+      </c>
+      <c r="D62" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="B63" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C63" s="12">
+        <v>10</v>
+      </c>
+      <c r="D63" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="B64" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C64" s="12">
+        <v>10</v>
+      </c>
+      <c r="D64" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B65" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C65" s="12">
+        <v>10</v>
+      </c>
+      <c r="D65" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B66" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C66" s="12">
+        <v>10</v>
+      </c>
+      <c r="D66" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B67" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C67" s="13">
+        <v>22.9</v>
+      </c>
+      <c r="D67" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B68" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="C68" s="12">
+        <v>60</v>
+      </c>
+      <c r="D68" s="11"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B69" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="C69" s="12">
+        <v>60</v>
+      </c>
+      <c r="D69" s="11"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="C70" s="12">
+        <v>60</v>
+      </c>
+      <c r="D70" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="C71" s="12">
+        <v>10</v>
+      </c>
+      <c r="D71" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B72" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C72" s="12">
+        <v>10</v>
+      </c>
+      <c r="D72" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="B73" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C73" s="12">
+        <v>10</v>
+      </c>
+      <c r="D73" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B74" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C74" s="12">
+        <v>10</v>
+      </c>
+      <c r="D74" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="B75" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="C75" s="12">
+        <v>10</v>
+      </c>
+      <c r="D75" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B76" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C76" s="12">
+        <v>10</v>
+      </c>
+      <c r="D76" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B77" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C77" s="12">
+        <v>10</v>
+      </c>
+      <c r="D77" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B78" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="C78" s="12">
+        <v>10</v>
+      </c>
+      <c r="D78" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="B79" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="C79" s="12">
+        <v>10</v>
+      </c>
+      <c r="D79" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B80" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="C80" s="12">
+        <v>60</v>
+      </c>
+      <c r="D80" s="11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B81" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C81" s="12">
+        <v>10</v>
+      </c>
+      <c r="D81" s="11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="B82" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="C82" s="12">
+        <v>10</v>
+      </c>
+      <c r="D82" s="11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="B83" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="C83" s="12">
+        <v>10</v>
+      </c>
+      <c r="D83" s="11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="B84" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="C84" s="12">
+        <v>10</v>
+      </c>
+      <c r="D84" s="11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="B85" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="C85" s="12">
+        <v>10</v>
+      </c>
+      <c r="D85" s="11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="B86" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C86" s="12">
+        <v>10</v>
+      </c>
+      <c r="D86" s="11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="B87" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="C87" s="12">
+        <v>10</v>
+      </c>
+      <c r="D87" s="11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B88" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="C88" s="12">
+        <v>60</v>
+      </c>
+      <c r="D88" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B89" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="C89" s="12">
+        <v>10</v>
+      </c>
+      <c r="D89" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B90" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="C90" s="13">
+        <v>22.9</v>
+      </c>
+      <c r="D90" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B91" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="C91" s="13">
+        <v>22.9</v>
+      </c>
+      <c r="D91" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B92" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="C92" s="12">
+        <v>60</v>
+      </c>
+      <c r="D92" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B93" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="C93" s="12">
+        <v>10</v>
+      </c>
+      <c r="D93" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="B94" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="C94" s="12">
+        <v>10</v>
+      </c>
+      <c r="D94" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="B95" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="C95" s="12">
+        <v>10</v>
+      </c>
+      <c r="D95" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="B96" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="C96" s="12">
+        <v>10</v>
+      </c>
+      <c r="D96" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="B97" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="C97" s="12">
+        <v>10</v>
+      </c>
+      <c r="D97" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B98" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="C98" s="12">
+        <v>60</v>
+      </c>
+      <c r="D98" s="11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B99" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="C99" s="12">
+        <v>10</v>
+      </c>
+      <c r="D99" s="11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B100" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="C100" s="12">
+        <v>60</v>
+      </c>
+      <c r="D100" s="11"/>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B101" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="C101" s="12">
+        <v>60</v>
+      </c>
+      <c r="D101" s="11"/>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A102" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B102" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="C102" s="12">
+        <v>60</v>
+      </c>
+      <c r="D102" s="11"/>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A103" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B103" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="C103" s="12">
+        <v>60</v>
+      </c>
+      <c r="D103" s="11"/>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B104" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="C104" s="12">
+        <v>60</v>
+      </c>
+      <c r="D104" s="11"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B105" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="C105" s="12">
+        <v>60</v>
+      </c>
+      <c r="D105" s="11"/>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A106" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B106" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="C106" s="12">
+        <v>60</v>
+      </c>
+      <c r="D106" s="11"/>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A107" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B107" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="C107" s="12">
+        <v>10</v>
+      </c>
+      <c r="D107" s="11" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A108" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B108" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="C108" s="13">
+        <v>22.9</v>
+      </c>
+      <c r="D108" s="11" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A109" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B109" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="C109" s="12">
+        <v>60</v>
+      </c>
+      <c r="D109" s="11" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A110" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="B110" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="C110" s="12">
+        <v>10</v>
+      </c>
+      <c r="D110" s="11" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A111" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="B111" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="C111" s="12">
+        <v>10</v>
+      </c>
+      <c r="D111" s="11" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A112" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="B112" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="C112" s="13">
+        <v>22.9</v>
+      </c>
+      <c r="D112" s="11" t="s">
+        <v>167</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
3.3b/3.3/3.4/5 fixes: real power not energy, SE/M consumption rule, fixed KWH allocation, 3.4 commits native captures, CYMDIST report+verify buttons
</commit_message>
<xml_diff>
--- a/data/input/common/medidoralimentador/medidoralimentador.xlsx
+++ b/data/input/common/medidoralimentador/medidoralimentador.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\ELDICA\RECYM\data\input\common\medidoralimentador\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB03DE83-0666-43EF-8FDD-5B65D28DE93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A149F706-61B1-4A45-AC34-65920401CFD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0537D3D3-A7EC-4918-978F-ABDC6DEFE1BE}"/>
+    <workbookView xWindow="-100" yWindow="0" windowWidth="12820" windowHeight="15370" xr2:uid="{0537D3D3-A7EC-4918-978F-ABDC6DEFE1BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="182">
   <si>
     <t>Medidor</t>
   </si>
@@ -564,6 +564,24 @@
   </si>
   <si>
     <t xml:space="preserve">CHN201   </t>
+  </si>
+  <si>
+    <t>IN111</t>
+  </si>
+  <si>
+    <t>IN111_V18 Y IN111_V119</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>TA225</t>
+  </si>
+  <si>
+    <t>L-TA225</t>
+  </si>
+  <si>
+    <t>TA</t>
   </si>
 </sst>
 </file>
@@ -621,7 +639,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -644,6 +662,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -654,25 +683,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -685,6 +705,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1021,1479 +1050,1507 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{316871D9-CF50-4EFA-B4A9-0D945CB9EBBB}">
-  <dimension ref="A2:D112"/>
+  <dimension ref="A2:D114"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" style="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="4">
-        <v>60</v>
-      </c>
-      <c r="D3" s="6"/>
+      <c r="C3" s="3">
+        <v>60</v>
+      </c>
+      <c r="D3" s="4"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="7">
-        <v>60</v>
-      </c>
-      <c r="D4" s="9"/>
+      <c r="C4" s="5">
+        <v>60</v>
+      </c>
+      <c r="D4" s="6"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4">
-        <v>10</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="C5" s="3">
+        <v>10</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="7">
-        <v>10</v>
-      </c>
-      <c r="D6" s="7" t="s">
+      <c r="C6" s="5">
+        <v>10</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="7">
-        <v>10</v>
-      </c>
-      <c r="D8" s="7" t="s">
+      <c r="C8" s="5">
+        <v>10</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="5" t="s">
+      <c r="A9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="4">
-        <v>60</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="C9" s="3">
+        <v>60</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="8" t="s">
+      <c r="A10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="7">
-        <v>10</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="C10" s="5">
+        <v>10</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="4">
-        <v>10</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="C11" s="3">
+        <v>10</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="7">
-        <v>10</v>
-      </c>
-      <c r="D12" s="7" t="s">
+      <c r="C12" s="5">
+        <v>10</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="4">
-        <v>10</v>
-      </c>
-      <c r="D13" s="4" t="s">
+      <c r="C13" s="3">
+        <v>10</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="7">
-        <v>10</v>
-      </c>
-      <c r="D14" s="7" t="s">
+      <c r="C14" s="5">
+        <v>10</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15" s="5" t="s">
+      <c r="A15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="4">
-        <v>60</v>
-      </c>
-      <c r="D15" s="4" t="s">
+      <c r="C15" s="3">
+        <v>60</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="8" t="s">
+      <c r="A16" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="7">
-        <v>10</v>
-      </c>
-      <c r="D16" s="7" t="s">
+      <c r="C16" s="5">
+        <v>10</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="4">
-        <v>10</v>
-      </c>
-      <c r="D17" s="4" t="s">
+      <c r="C17" s="3">
+        <v>10</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="7">
-        <v>10</v>
-      </c>
-      <c r="D18" s="7" t="s">
+      <c r="C18" s="5">
+        <v>10</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="4">
-        <v>10</v>
-      </c>
-      <c r="D19" s="4" t="s">
+      <c r="C19" s="3">
+        <v>10</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="7">
-        <v>10</v>
-      </c>
-      <c r="D20" s="7" t="s">
+      <c r="C20" s="5">
+        <v>10</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="4">
-        <v>10</v>
-      </c>
-      <c r="D21" s="4" t="s">
+      <c r="C21" s="3">
+        <v>10</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B23" s="5" t="s">
+      <c r="A23" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="7">
-        <v>60</v>
-      </c>
-      <c r="D24" s="7" t="s">
+      <c r="C24" s="5">
+        <v>60</v>
+      </c>
+      <c r="D24" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B25" s="5" t="s">
+      <c r="A25" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="4">
-        <v>60</v>
-      </c>
-      <c r="D25" s="4" t="s">
+      <c r="C25" s="3">
+        <v>60</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B27" s="5" t="s">
+      <c r="A27" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C27" s="4">
-        <v>10</v>
-      </c>
-      <c r="D27" s="4" t="s">
+      <c r="C27" s="3">
+        <v>10</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C28" s="7">
-        <v>10</v>
-      </c>
-      <c r="D28" s="7" t="s">
+      <c r="C28" s="5">
+        <v>10</v>
+      </c>
+      <c r="D28" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C29" s="4">
-        <v>10</v>
-      </c>
-      <c r="D29" s="4" t="s">
+      <c r="C29" s="3">
+        <v>10</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B30" s="8" t="s">
+      <c r="A30" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C30" s="7">
-        <v>60</v>
-      </c>
-      <c r="D30" s="7" t="s">
+      <c r="C30" s="5">
+        <v>60</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" s="6"/>
-      <c r="B31" s="5" t="s">
+      <c r="A31" s="4"/>
+      <c r="B31" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" s="7" t="s">
+      <c r="A32" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" s="6"/>
-      <c r="B33" s="5" t="s">
+      <c r="A33" s="4"/>
+      <c r="B33" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C34" s="7">
-        <v>10</v>
-      </c>
-      <c r="D34" s="7" t="s">
+      <c r="C34" s="5">
+        <v>10</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C35" s="4">
-        <v>10</v>
-      </c>
-      <c r="D35" s="4" t="s">
+      <c r="C35" s="3">
+        <v>10</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B36" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C36" s="7">
-        <v>60</v>
-      </c>
-      <c r="D36" s="9"/>
+      <c r="A36" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C36" s="5">
+        <v>60</v>
+      </c>
+      <c r="D36" s="6"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C37" s="4">
-        <v>60</v>
-      </c>
-      <c r="D37" s="6"/>
+      <c r="C37" s="3">
+        <v>60</v>
+      </c>
+      <c r="D37" s="4"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A38" s="7" t="s">
+      <c r="A38" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B39" s="5" t="s">
+      <c r="A39" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B39" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="D39" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" s="7" t="s">
+      <c r="A40" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C40" s="7">
+      <c r="C40" s="5">
         <v>220</v>
       </c>
-      <c r="D40" s="9"/>
+      <c r="D40" s="6"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C41" s="4">
+      <c r="C41" s="3">
         <v>220</v>
       </c>
-      <c r="D41" s="6"/>
+      <c r="D41" s="4"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A42" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B42" s="8" t="s">
+      <c r="A42" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B42" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C42" s="7">
+      <c r="C42" s="5">
         <v>220</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="D42" s="5" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C43" s="4">
-        <v>60</v>
-      </c>
-      <c r="D43" s="6"/>
+      <c r="C43" s="3">
+        <v>60</v>
+      </c>
+      <c r="D43" s="4"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A44" s="7" t="s">
+      <c r="A44" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C44" s="7" t="s">
+      <c r="C44" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D44" s="9"/>
+      <c r="D44" s="6"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A45" s="6"/>
-      <c r="B45" s="5" t="s">
+      <c r="A45" s="4"/>
+      <c r="B45" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A46" s="9"/>
-      <c r="B46" s="8" t="s">
+      <c r="A46" s="6"/>
+      <c r="B46" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C46" s="9"/>
-      <c r="D46" s="9"/>
+      <c r="C46" s="6"/>
+      <c r="D46" s="6"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A47" s="6"/>
-      <c r="B47" s="5" t="s">
+      <c r="A47" s="4"/>
+      <c r="B47" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A48" s="9"/>
-      <c r="B48" s="8" t="s">
+      <c r="A48" s="6"/>
+      <c r="B48" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C48" s="9"/>
-      <c r="D48" s="9"/>
+      <c r="C48" s="6"/>
+      <c r="D48" s="6"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A49" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B49" s="5" t="s">
+      <c r="A49" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B49" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C49" s="4">
-        <v>10</v>
-      </c>
-      <c r="D49" s="4" t="s">
+      <c r="C49" s="3">
+        <v>10</v>
+      </c>
+      <c r="D49" s="3" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A50" s="7" t="s">
+      <c r="A50" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B50" s="8" t="s">
+      <c r="B50" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C50" s="7">
-        <v>10</v>
-      </c>
-      <c r="D50" s="7" t="s">
+      <c r="C50" s="5">
+        <v>10</v>
+      </c>
+      <c r="D50" s="5" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A51" s="10"/>
-      <c r="B51" s="5" t="s">
+      <c r="A51" s="7"/>
+      <c r="B51" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A52" s="10"/>
-      <c r="B52" s="8" t="s">
+      <c r="A52" s="7"/>
+      <c r="B52" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C52" s="9"/>
-      <c r="D52" s="9"/>
+      <c r="C52" s="6"/>
+      <c r="D52" s="6"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A53" s="11" t="s">
+      <c r="A53" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B53" s="11" t="s">
+      <c r="B53" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="C53" s="12">
-        <v>60</v>
-      </c>
-      <c r="D53" s="11"/>
+      <c r="C53" s="9">
+        <v>60</v>
+      </c>
+      <c r="D53" s="8"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A54" s="11" t="s">
+      <c r="A54" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B54" s="11" t="s">
+      <c r="B54" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C54" s="12">
-        <v>60</v>
-      </c>
-      <c r="D54" s="11"/>
+      <c r="C54" s="9">
+        <v>60</v>
+      </c>
+      <c r="D54" s="8"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A55" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B55" s="11" t="s">
+      <c r="A55" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B55" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="C55" s="12">
-        <v>60</v>
-      </c>
-      <c r="D55" s="11" t="s">
+      <c r="C55" s="9">
+        <v>60</v>
+      </c>
+      <c r="D55" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A56" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B56" s="11" t="s">
+      <c r="A56" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B56" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="C56" s="12">
-        <v>10</v>
-      </c>
-      <c r="D56" s="11" t="s">
+      <c r="C56" s="9">
+        <v>10</v>
+      </c>
+      <c r="D56" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A57" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B57" s="11" t="s">
+      <c r="A57" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B57" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C57" s="13">
+      <c r="C57" s="10">
         <v>22.9</v>
       </c>
-      <c r="D57" s="11" t="s">
+      <c r="D57" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A58" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B58" s="11" t="s">
+      <c r="A58" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B58" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="C58" s="12">
-        <v>60</v>
-      </c>
-      <c r="D58" s="11" t="s">
+      <c r="C58" s="9">
+        <v>60</v>
+      </c>
+      <c r="D58" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A59" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B59" s="11" t="s">
+      <c r="A59" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B59" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="C59" s="12">
-        <v>10</v>
-      </c>
-      <c r="D59" s="11" t="s">
+      <c r="C59" s="9">
+        <v>10</v>
+      </c>
+      <c r="D59" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A60" s="11" t="s">
+      <c r="A60" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B60" s="11" t="s">
+      <c r="B60" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C60" s="12">
-        <v>10</v>
-      </c>
-      <c r="D60" s="11" t="s">
+      <c r="C60" s="9">
+        <v>10</v>
+      </c>
+      <c r="D60" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A61" s="11" t="s">
+      <c r="A61" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="B61" s="11" t="s">
+      <c r="B61" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="C61" s="12">
-        <v>10</v>
-      </c>
-      <c r="D61" s="11" t="s">
+      <c r="C61" s="9">
+        <v>10</v>
+      </c>
+      <c r="D61" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A62" s="11" t="s">
+      <c r="A62" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B62" s="11" t="s">
+      <c r="B62" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="C62" s="12">
-        <v>10</v>
-      </c>
-      <c r="D62" s="11" t="s">
+      <c r="C62" s="9">
+        <v>10</v>
+      </c>
+      <c r="D62" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A63" s="11" t="s">
+      <c r="A63" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B63" s="11" t="s">
+      <c r="B63" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="C63" s="12">
-        <v>10</v>
-      </c>
-      <c r="D63" s="11" t="s">
+      <c r="C63" s="9">
+        <v>10</v>
+      </c>
+      <c r="D63" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A64" s="11" t="s">
+      <c r="A64" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="B64" s="11" t="s">
+      <c r="B64" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="C64" s="12">
-        <v>10</v>
-      </c>
-      <c r="D64" s="11" t="s">
+      <c r="C64" s="9">
+        <v>10</v>
+      </c>
+      <c r="D64" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A65" s="11" t="s">
+      <c r="A65" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="B65" s="11" t="s">
+      <c r="B65" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="C65" s="12">
-        <v>10</v>
-      </c>
-      <c r="D65" s="11" t="s">
+      <c r="C65" s="9">
+        <v>10</v>
+      </c>
+      <c r="D65" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A66" s="11" t="s">
+      <c r="A66" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B66" s="11" t="s">
+      <c r="B66" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="C66" s="12">
-        <v>10</v>
-      </c>
-      <c r="D66" s="11" t="s">
+      <c r="C66" s="9">
+        <v>10</v>
+      </c>
+      <c r="D66" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A67" s="11" t="s">
+      <c r="A67" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="B67" s="11" t="s">
+      <c r="B67" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="C67" s="13">
+      <c r="C67" s="10">
         <v>22.9</v>
       </c>
-      <c r="D67" s="11" t="s">
+      <c r="D67" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A68" s="11" t="s">
+      <c r="A68" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B68" s="11" t="s">
+      <c r="B68" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="C68" s="12">
-        <v>60</v>
-      </c>
-      <c r="D68" s="11"/>
+      <c r="C68" s="9">
+        <v>60</v>
+      </c>
+      <c r="D68" s="8"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A69" s="11" t="s">
+      <c r="A69" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B69" s="11" t="s">
+      <c r="B69" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="C69" s="12">
-        <v>60</v>
-      </c>
-      <c r="D69" s="11"/>
+      <c r="C69" s="9">
+        <v>60</v>
+      </c>
+      <c r="D69" s="8"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A70" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B70" s="11" t="s">
+      <c r="A70" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B70" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="C70" s="12">
-        <v>60</v>
-      </c>
-      <c r="D70" s="11" t="s">
+      <c r="C70" s="9">
+        <v>60</v>
+      </c>
+      <c r="D70" s="8" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A71" s="11" t="s">
+      <c r="A71" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="B71" s="11" t="s">
+      <c r="B71" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="C71" s="12">
-        <v>10</v>
-      </c>
-      <c r="D71" s="11" t="s">
+      <c r="C71" s="9">
+        <v>10</v>
+      </c>
+      <c r="D71" s="8" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A72" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B72" s="11" t="s">
+      <c r="A72" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B72" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="C72" s="12">
-        <v>10</v>
-      </c>
-      <c r="D72" s="11" t="s">
+      <c r="C72" s="9">
+        <v>10</v>
+      </c>
+      <c r="D72" s="8" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A73" s="11" t="s">
+      <c r="A73" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="B73" s="11" t="s">
+      <c r="B73" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="C73" s="12">
-        <v>10</v>
-      </c>
-      <c r="D73" s="11" t="s">
+      <c r="C73" s="9">
+        <v>10</v>
+      </c>
+      <c r="D73" s="8" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A74" s="11" t="s">
+      <c r="A74" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="B74" s="11" t="s">
+      <c r="B74" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="C74" s="12">
-        <v>10</v>
-      </c>
-      <c r="D74" s="11" t="s">
+      <c r="C74" s="9">
+        <v>10</v>
+      </c>
+      <c r="D74" s="8" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A75" s="11" t="s">
+      <c r="A75" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="B75" s="11" t="s">
+      <c r="B75" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="C75" s="12">
-        <v>10</v>
-      </c>
-      <c r="D75" s="11" t="s">
+      <c r="C75" s="9">
+        <v>10</v>
+      </c>
+      <c r="D75" s="8" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A76" s="11" t="s">
+      <c r="A76" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="B76" s="11" t="s">
+      <c r="B76" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="C76" s="12">
-        <v>10</v>
-      </c>
-      <c r="D76" s="11" t="s">
+      <c r="C76" s="9">
+        <v>10</v>
+      </c>
+      <c r="D76" s="8" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A77" s="11" t="s">
+      <c r="A77" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="B77" s="11" t="s">
+      <c r="B77" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="C77" s="12">
-        <v>10</v>
-      </c>
-      <c r="D77" s="11" t="s">
+      <c r="C77" s="9">
+        <v>10</v>
+      </c>
+      <c r="D77" s="8" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A78" s="11" t="s">
+      <c r="A78" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="B78" s="11" t="s">
+      <c r="B78" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="C78" s="12">
-        <v>10</v>
-      </c>
-      <c r="D78" s="11" t="s">
+      <c r="C78" s="9">
+        <v>10</v>
+      </c>
+      <c r="D78" s="8" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A79" s="11" t="s">
+      <c r="A79" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="B79" s="11" t="s">
+      <c r="B79" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="C79" s="12">
-        <v>10</v>
-      </c>
-      <c r="D79" s="11" t="s">
+      <c r="C79" s="9">
+        <v>10</v>
+      </c>
+      <c r="D79" s="8" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A80" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B80" s="11" t="s">
+      <c r="A80" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B80" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="C80" s="12">
-        <v>60</v>
-      </c>
-      <c r="D80" s="11" t="s">
+      <c r="C80" s="9">
+        <v>60</v>
+      </c>
+      <c r="D80" s="8" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A81" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B81" s="11" t="s">
+      <c r="A81" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B81" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="C81" s="12">
-        <v>10</v>
-      </c>
-      <c r="D81" s="11" t="s">
+      <c r="C81" s="9">
+        <v>10</v>
+      </c>
+      <c r="D81" s="8" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A82" s="11" t="s">
+      <c r="A82" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="B82" s="11" t="s">
+      <c r="B82" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="C82" s="12">
-        <v>10</v>
-      </c>
-      <c r="D82" s="11" t="s">
+      <c r="C82" s="9">
+        <v>10</v>
+      </c>
+      <c r="D82" s="8" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A83" s="11" t="s">
+      <c r="A83" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="B83" s="11" t="s">
+      <c r="B83" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="C83" s="12">
-        <v>10</v>
-      </c>
-      <c r="D83" s="11" t="s">
+      <c r="C83" s="9">
+        <v>10</v>
+      </c>
+      <c r="D83" s="8" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A84" s="11" t="s">
+      <c r="A84" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="B84" s="11" t="s">
+      <c r="B84" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="C84" s="12">
-        <v>10</v>
-      </c>
-      <c r="D84" s="11" t="s">
+      <c r="C84" s="9">
+        <v>10</v>
+      </c>
+      <c r="D84" s="8" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A85" s="11" t="s">
+      <c r="A85" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="B85" s="11" t="s">
+      <c r="B85" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="C85" s="12">
-        <v>10</v>
-      </c>
-      <c r="D85" s="11" t="s">
+      <c r="C85" s="9">
+        <v>10</v>
+      </c>
+      <c r="D85" s="8" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A86" s="11" t="s">
+      <c r="A86" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="B86" s="11" t="s">
+      <c r="B86" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="C86" s="12">
-        <v>10</v>
-      </c>
-      <c r="D86" s="11" t="s">
+      <c r="C86" s="9">
+        <v>10</v>
+      </c>
+      <c r="D86" s="8" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A87" s="11" t="s">
+      <c r="A87" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B87" s="11" t="s">
+      <c r="B87" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="C87" s="12">
-        <v>10</v>
-      </c>
-      <c r="D87" s="11" t="s">
+      <c r="C87" s="9">
+        <v>10</v>
+      </c>
+      <c r="D87" s="8" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A88" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B88" s="11" t="s">
+      <c r="A88" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B88" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="C88" s="12">
-        <v>60</v>
-      </c>
-      <c r="D88" s="11" t="s">
+      <c r="C88" s="9">
+        <v>60</v>
+      </c>
+      <c r="D88" s="8" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A89" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B89" s="11" t="s">
+      <c r="A89" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B89" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="C89" s="12">
-        <v>10</v>
-      </c>
-      <c r="D89" s="11" t="s">
+      <c r="C89" s="9">
+        <v>10</v>
+      </c>
+      <c r="D89" s="8" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A90" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B90" s="11" t="s">
+      <c r="A90" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B90" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="C90" s="13">
+      <c r="C90" s="10">
         <v>22.9</v>
       </c>
-      <c r="D90" s="11" t="s">
+      <c r="D90" s="8" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A91" s="11" t="s">
+      <c r="A91" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="B91" s="11" t="s">
+      <c r="B91" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="C91" s="13">
+      <c r="C91" s="10">
         <v>22.9</v>
       </c>
-      <c r="D91" s="11" t="s">
+      <c r="D91" s="8" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A92" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B92" s="11" t="s">
+      <c r="A92" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B92" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="C92" s="12">
-        <v>60</v>
-      </c>
-      <c r="D92" s="11" t="s">
+      <c r="C92" s="9">
+        <v>60</v>
+      </c>
+      <c r="D92" s="8" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A93" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B93" s="11" t="s">
+      <c r="A93" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B93" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="C93" s="12">
-        <v>10</v>
-      </c>
-      <c r="D93" s="11" t="s">
+      <c r="C93" s="9">
+        <v>10</v>
+      </c>
+      <c r="D93" s="8" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A94" s="11" t="s">
+      <c r="A94" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="B94" s="11" t="s">
+      <c r="B94" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="C94" s="12">
-        <v>10</v>
-      </c>
-      <c r="D94" s="11" t="s">
+      <c r="C94" s="9">
+        <v>10</v>
+      </c>
+      <c r="D94" s="8" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A95" s="11" t="s">
+      <c r="A95" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="B95" s="11" t="s">
+      <c r="B95" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="C95" s="12">
-        <v>10</v>
-      </c>
-      <c r="D95" s="11" t="s">
+      <c r="C95" s="9">
+        <v>10</v>
+      </c>
+      <c r="D95" s="8" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A96" s="11" t="s">
+      <c r="A96" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="B96" s="11" t="s">
+      <c r="B96" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="C96" s="12">
-        <v>10</v>
-      </c>
-      <c r="D96" s="11" t="s">
+      <c r="C96" s="9">
+        <v>10</v>
+      </c>
+      <c r="D96" s="8" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A97" s="11" t="s">
+      <c r="A97" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="B97" s="11" t="s">
+      <c r="B97" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C97" s="12">
-        <v>10</v>
-      </c>
-      <c r="D97" s="11" t="s">
+      <c r="C97" s="9">
+        <v>10</v>
+      </c>
+      <c r="D97" s="8" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A98" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B98" s="11" t="s">
+      <c r="A98" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B98" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="C98" s="12">
-        <v>60</v>
-      </c>
-      <c r="D98" s="11" t="s">
+      <c r="C98" s="9">
+        <v>60</v>
+      </c>
+      <c r="D98" s="8" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A99" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B99" s="11" t="s">
+      <c r="A99" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B99" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="C99" s="12">
-        <v>10</v>
-      </c>
-      <c r="D99" s="11" t="s">
+      <c r="C99" s="9">
+        <v>10</v>
+      </c>
+      <c r="D99" s="8" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A100" s="11" t="s">
+      <c r="A100" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B100" s="11" t="s">
+      <c r="B100" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="C100" s="12">
-        <v>60</v>
-      </c>
-      <c r="D100" s="11"/>
+      <c r="C100" s="9">
+        <v>60</v>
+      </c>
+      <c r="D100" s="8"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A101" s="11" t="s">
+      <c r="A101" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B101" s="11" t="s">
+      <c r="B101" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="C101" s="12">
-        <v>60</v>
-      </c>
-      <c r="D101" s="11"/>
+      <c r="C101" s="9">
+        <v>60</v>
+      </c>
+      <c r="D101" s="8"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A102" s="11" t="s">
+      <c r="A102" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B102" s="11" t="s">
+      <c r="B102" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="C102" s="12">
-        <v>60</v>
-      </c>
-      <c r="D102" s="11"/>
+      <c r="C102" s="9">
+        <v>60</v>
+      </c>
+      <c r="D102" s="8"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A103" s="11" t="s">
+      <c r="A103" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B103" s="11" t="s">
+      <c r="B103" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="C103" s="12">
-        <v>60</v>
-      </c>
-      <c r="D103" s="11"/>
+      <c r="C103" s="9">
+        <v>60</v>
+      </c>
+      <c r="D103" s="8"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A104" s="11" t="s">
+      <c r="A104" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B104" s="11" t="s">
+      <c r="B104" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="C104" s="12">
-        <v>60</v>
-      </c>
-      <c r="D104" s="11"/>
+      <c r="C104" s="9">
+        <v>60</v>
+      </c>
+      <c r="D104" s="8"/>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A105" s="11" t="s">
+      <c r="A105" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B105" s="11" t="s">
+      <c r="B105" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="C105" s="12">
-        <v>60</v>
-      </c>
-      <c r="D105" s="11"/>
+      <c r="C105" s="9">
+        <v>60</v>
+      </c>
+      <c r="D105" s="8"/>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A106" s="11" t="s">
+      <c r="A106" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B106" s="11" t="s">
+      <c r="B106" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="C106" s="12">
-        <v>60</v>
-      </c>
-      <c r="D106" s="11"/>
+      <c r="C106" s="9">
+        <v>60</v>
+      </c>
+      <c r="D106" s="8"/>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A107" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B107" s="11" t="s">
+      <c r="A107" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B107" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="C107" s="12">
-        <v>10</v>
-      </c>
-      <c r="D107" s="11" t="s">
+      <c r="C107" s="9">
+        <v>10</v>
+      </c>
+      <c r="D107" s="8" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A108" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B108" s="11" t="s">
+      <c r="A108" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B108" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="C108" s="13">
+      <c r="C108" s="10">
         <v>22.9</v>
       </c>
-      <c r="D108" s="11" t="s">
+      <c r="D108" s="8" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A109" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B109" s="11" t="s">
+      <c r="A109" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B109" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="C109" s="12">
-        <v>60</v>
-      </c>
-      <c r="D109" s="11" t="s">
+      <c r="C109" s="9">
+        <v>60</v>
+      </c>
+      <c r="D109" s="8" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A110" s="11" t="s">
+      <c r="A110" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="B110" s="11" t="s">
+      <c r="B110" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="C110" s="12">
-        <v>10</v>
-      </c>
-      <c r="D110" s="11" t="s">
+      <c r="C110" s="9">
+        <v>10</v>
+      </c>
+      <c r="D110" s="8" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A111" s="11" t="s">
+      <c r="A111" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="B111" s="11" t="s">
+      <c r="B111" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="C111" s="12">
-        <v>10</v>
-      </c>
-      <c r="D111" s="11" t="s">
+      <c r="C111" s="9">
+        <v>10</v>
+      </c>
+      <c r="D111" s="8" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A112" s="11" t="s">
+      <c r="A112" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="B112" s="11" t="s">
+      <c r="B112" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="C112" s="13">
+      <c r="C112" s="10">
         <v>22.9</v>
       </c>
-      <c r="D112" s="11" t="s">
+      <c r="D112" s="8" t="s">
         <v>167</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A113" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="B113" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="C113" s="12">
+        <v>10</v>
+      </c>
+      <c r="D113" s="11" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A114" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="B114" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="C114" s="12">
+        <v>22.9</v>
+      </c>
+      <c r="D114" s="11" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>